<commit_message>
Update: Code changes from Bob IDE
</commit_message>
<xml_diff>
--- a/Learning.xlsx
+++ b/Learning.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Bob\workspace\ci-mgmt-app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E30EF27E-8BEB-4984-8FE2-33A03D516D3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55829ABA-6B61-47F5-9ED7-8781394FE9E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>NEXT STEPS (Choose One)
 Option A: Deploy Now (Recommended)
@@ -133,9 +133,6 @@
       <t xml:space="preserve">
 cd backend; mvn spring-boot:run</t>
     </r>
-  </si>
-  <si>
-    <t>eaartyadav@gmail.com/</t>
   </si>
   <si>
     <t>echotababu@gmail.com/echotababu@start001</t>
@@ -284,12 +281,30 @@
   <si>
     <t>https://neon.tech</t>
   </si>
+  <si>
+    <t>eaartiyadav@gmail.com/</t>
+  </si>
+  <si>
+    <t>http://localhost:5173/</t>
+  </si>
+  <si>
+    <t>admin@cims.com/Admin@123</t>
+  </si>
+  <si>
+    <t>http://192.168.0.211:5173</t>
+  </si>
+  <si>
+    <t>home</t>
+  </si>
+  <si>
+    <t>admin/admin001</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -334,6 +349,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -362,7 +385,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -380,6 +403,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -661,153 +685,173 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="81.109375" customWidth="1"/>
     <col min="3" max="3" width="28.77734375" customWidth="1"/>
-    <col min="5" max="5" width="27.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="47.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B2" s="7" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B1" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B3" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B4" s="7"/>
+      <c r="E4" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B5" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B6" s="7" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B3" s="7"/>
-    </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B4" s="8" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B5" s="7" t="s">
+      <c r="E6" s="9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B7" s="7" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B6" s="7" t="s">
+      <c r="C7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+      <c r="B8" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C8" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="2:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="B7" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B8" s="7"/>
-    </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B10" t="s">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B9" s="7"/>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B11" t="s">
         <v>1</v>
       </c>
-      <c r="E10" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B11" s="1" t="s">
+    </row>
+    <row r="12" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B12" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E11" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B12" s="1"/>
-      <c r="E12" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="13" spans="2:5" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B13" s="1" t="s">
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B13" s="1"/>
+    </row>
+    <row r="14" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B14" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E13" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="E14" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B15" t="s">
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B16" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="2:3" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B17" s="1" t="s">
+    <row r="18" spans="2:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B18" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B19" t="s">
+    <row r="20" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B20" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B20" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="21" spans="2:3" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B21" s="4" t="s">
+    <row r="21" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B21" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B22" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B22" s="5" t="s">
+    <row r="23" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B23" s="5" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B23" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="24" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
-        <v>9</v>
-      </c>
-      <c r="C24" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
+        <v>9</v>
+      </c>
+      <c r="C25" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="26" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B26" t="s">
         <v>10</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C26" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="27" spans="2:3" ht="72" x14ac:dyDescent="0.3">
-      <c r="B27" s="1" t="s">
+    <row r="28" spans="2:3" ht="72" x14ac:dyDescent="0.3">
+      <c r="B28" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C28" t="s">
         <v>21</v>
-      </c>
-      <c r="C27" t="s">
-        <v>22</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E10" r:id="rId1" xr:uid="{536EDB48-6B0E-4AC1-89CE-93C7AE78B8E4}"/>
-    <hyperlink ref="E11" r:id="rId2" xr:uid="{C012FC16-5930-4AB6-AD8E-40283780F4B2}"/>
-    <hyperlink ref="E12" r:id="rId3" xr:uid="{9C428AA7-AC03-47EE-8846-5D9DB0E9FC40}"/>
-    <hyperlink ref="E13" r:id="rId4" xr:uid="{4CE4418D-B483-4B94-9549-589B7F2D4708}"/>
-    <hyperlink ref="E14" r:id="rId5" xr:uid="{BFC4A828-184F-4B54-9FC1-8A8A65FD188F}"/>
-    <hyperlink ref="B4" r:id="rId6" xr:uid="{78F88DDC-8A28-42B2-9AB0-ECEF5E8B1923}"/>
+    <hyperlink ref="E3" r:id="rId1" xr:uid="{536EDB48-6B0E-4AC1-89CE-93C7AE78B8E4}"/>
+    <hyperlink ref="E4" r:id="rId2" xr:uid="{C012FC16-5930-4AB6-AD8E-40283780F4B2}"/>
+    <hyperlink ref="E5" r:id="rId3" xr:uid="{9C428AA7-AC03-47EE-8846-5D9DB0E9FC40}"/>
+    <hyperlink ref="E6" r:id="rId4" xr:uid="{4CE4418D-B483-4B94-9549-589B7F2D4708}"/>
+    <hyperlink ref="E7" r:id="rId5" xr:uid="{BFC4A828-184F-4B54-9FC1-8A8A65FD188F}"/>
+    <hyperlink ref="B5" r:id="rId6" xr:uid="{78F88DDC-8A28-42B2-9AB0-ECEF5E8B1923}"/>
+    <hyperlink ref="B1" r:id="rId7" xr:uid="{8E62CC93-7E2A-4921-8888-FE68D2F5C980}"/>
+    <hyperlink ref="C1" r:id="rId8" xr:uid="{EB4B9F32-FC8E-436A-9D8B-694F37AEDB43}"/>
+    <hyperlink ref="B2" r:id="rId9" xr:uid="{63C45EA7-4228-4057-90D3-6CB84D992E1D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -823,7 +867,7 @@
   <sheetData>
     <row r="2" spans="2:2" ht="409.6" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -846,7 +890,7 @@
     </row>
     <row r="4" spans="2:2" ht="172.8" x14ac:dyDescent="0.3">
       <c r="B4" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>